<commit_message>
replacing template file with one that does not have enzyme yield
</commit_message>
<xml_diff>
--- a/public/downloads/kinetic_assay_single_variant_template.xlsx
+++ b/public/downloads/kinetic_assay_single_variant_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\D2D-Cure\Website\Data Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lhynard\Documents\D2D-Cure\Website\Data Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA13B90C-60BD-40C4-AAAF-2EB177400A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B45E89A-717B-44A0-B3F5-7E018E9D8805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="0" windowWidth="26505" windowHeight="15750" xr2:uid="{CB8ED20E-9F28-4ABC-8126-9A5428C6413A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{CB8ED20E-9F28-4ABC-8126-9A5428C6413A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>A</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t>Column</t>
-  </si>
-  <si>
-    <t>Yield</t>
   </si>
   <si>
     <r>
@@ -167,16 +164,16 @@
     <t>420 nm over time</t>
   </si>
   <si>
-    <t>(mg/mL)</t>
-  </si>
-  <si>
-    <t>3. Enter the slopes for each well in the correct row and column to the left.</t>
-  </si>
-  <si>
-    <t>4. Select the units used by your instrument for slope from the dropdown.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Record the dates of purification and analysis above.  </t>
+    <t xml:space="preserve">1. Above, select or enter the dilution (usually 10× or 100×) of your enzyme solution used in the assay. </t>
+  </si>
+  <si>
+    <t>2. To the left, enter the slopes for each well in the correct row and column.</t>
+  </si>
+  <si>
+    <t>3. Select the units used by your instrument for slope from the dropdown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Above, record the dates of purification and analysis.  </t>
   </si>
   <si>
     <r>
@@ -187,7 +184,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">7. Be sure to save the file </t>
+      <t xml:space="preserve">5. Be sure to save the file </t>
     </r>
     <r>
       <rPr>
@@ -233,60 +230,14 @@
     </r>
   </si>
   <si>
-    <t>8. Ensure that Excel saved cells with scientific notation as numbers, not zeros.</t>
-  </si>
-  <si>
-    <t>1. Enter the yield (enzyme concentration) for your variant above.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">*If used, raw </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="subscript"/>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>280</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> values should be preadjusted for a path length of 1 cm. </t>
-    </r>
-  </si>
-  <si>
-    <t>5. Select the units used by your concentration assay from the dropdown.*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Select or enter the dilution (usually 10× or 100×) used in the assay above. </t>
+    <t>6. Ensure that Excel saved cells with scientific notation as numbers, not zeros.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -345,12 +296,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
@@ -359,30 +304,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF7030A0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF7030A0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7030A0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <vertAlign val="subscript"/>
       <sz val="11"/>
       <color rgb="FF7030A0"/>
       <name val="Calibri"/>
@@ -414,7 +335,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -588,22 +509,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -635,50 +545,34 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -719,9 +613,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -759,7 +653,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -865,7 +759,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1007,7 +901,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1025,69 +919,62 @@
   <sheetData>
     <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="27"/>
+      <c r="E1" s="28"/>
+      <c r="H1" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C2" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="32"/>
-      <c r="E1" s="33"/>
-      <c r="G1" s="17" t="s">
+      <c r="D2" s="25"/>
+      <c r="E2" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C2" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="18" t="s">
+      <c r="B3" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="17"/>
+      <c r="E3" s="18"/>
+      <c r="H3" s="14">
+        <v>10</v>
+      </c>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+    </row>
+    <row r="4" spans="1:10" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="A4" s="21"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="26"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="20"/>
-      <c r="E3" s="21"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="16">
-        <v>10</v>
-      </c>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-    </row>
-    <row r="4" spans="1:10" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A4" s="24"/>
-      <c r="B4" s="22"/>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -1101,7 +988,7 @@
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
       <c r="G5" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -1115,7 +1002,7 @@
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -1128,7 +1015,7 @@
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
-      <c r="G7" t="s">
+      <c r="G7" s="12" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1142,11 +1029,11 @@
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
-      <c r="G8" s="13" t="s">
+      <c r="G8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>0.92592592600000001</v>
       </c>
@@ -1156,8 +1043,8 @@
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
-      <c r="G9" s="14" t="s">
-        <v>29</v>
+      <c r="G9" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1171,10 +1058,10 @@
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="G10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>0.102880658</v>
       </c>
@@ -1184,9 +1071,6 @@
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
-      <c r="G11" s="1" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7">
@@ -1198,9 +1082,6 @@
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
-      <c r="G12" t="s">
-        <v>26</v>
-      </c>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
@@ -1209,10 +1090,8 @@
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
     </row>
-    <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A14" s="14" t="s">
-        <v>28</v>
-      </c>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="13"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
@@ -1221,25 +1100,22 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="J1:J2"/>
-    <mergeCell ref="H1:H2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C1:E1"/>
+    <mergeCell ref="H1:H2"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations disablePrompts="1" count="4">
     <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please enter a number greater than zero." sqref="C5:E12" xr:uid="{39023C31-5F86-42A7-9F0E-2A0526E36304}">
       <formula1>0</formula1>
       <formula2>9.99999999999999E+254</formula2>
     </dataValidation>
-    <dataValidation type="list" showInputMessage="1" errorTitle="Invalid value" error="You must select a value of 1× or 100× here." promptTitle="Dilution note" prompt="Typically, a value of 1× or 100× is entered here, but other dilutions are permissible." sqref="H3" xr:uid="{07532193-61B2-49D7-992D-2E69DD933868}">
+    <dataValidation type="list" showInputMessage="1" errorTitle="Invalid value" error="You must select a value of 1× or 100× here." promptTitle="Dilution note" prompt="Typically, a value of 10× or 100× is entered here, but other dilutions are permissible." sqref="H3" xr:uid="{07532193-61B2-49D7-992D-2E69DD933868}">
       <formula1>"10,100"</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please enter a valid date." sqref="I3:J3" xr:uid="{00DA71B4-1A95-4DB0-B7EE-9949BC233802}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please enter a valid date." sqref="J3 I3" xr:uid="{00DA71B4-1A95-4DB0-B7EE-9949BC233802}">
       <formula1>36892</formula1>
       <formula2>73415</formula2>
-    </dataValidation>
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="You must select a an option from the dropdown list." sqref="G2" xr:uid="{79B78625-270C-49F6-85C0-531CA5C893DE}">
-      <formula1>"A280*,(mg/mL),(uM),(mM),(M)"</formula1>
     </dataValidation>
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid units!" error="Please select the units for the slope from the list." promptTitle="(units)" prompt="Please select the units for the slope from the list." sqref="E2" xr:uid="{093563FB-F93C-490A-A2DA-2A6C44ADF49C}">
       <formula1>"(1/min),(1/s),(10^-3/min),(10^-3/s)"</formula1>

</xml_diff>